<commit_message>
feat: release v2.20.0 - D3-NET port calculation, DCS303/Modbus rules, Lingli section, and controller&pipe sync
</commit_message>
<xml_diff>
--- a/EQUIPMENT_Data.xlsx
+++ b/EQUIPMENT_Data.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9EF483C-5E4C-4DCA-A613-CC50AFC93250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20AE930-581C-456C-89EE-64F8ED51DB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7596" yWindow="168" windowWidth="15504" windowHeight="12240" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_units" sheetId="1" r:id="rId1"/>
-    <sheet name="controller" sheetId="5" r:id="rId2"/>
+    <sheet name="controller&amp;pipe" sheetId="5" r:id="rId2"/>
     <sheet name="outdoor_units" sheetId="2" r:id="rId3"/>
     <sheet name="indoor_units_SA only" sheetId="3" r:id="rId4"/>
     <sheet name="outdoor_units_SA only" sheetId="4" r:id="rId5"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3780" uniqueCount="623">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3803" uniqueCount="634">
   <si>
     <t>資料型態</t>
   </si>
@@ -2395,6 +2395,50 @@
   </si>
   <si>
     <t>RHF40VAVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DCPH01H</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>含Z-wave</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>伶俐智控管理器-住宅</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VRV分歧頭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KHRP26A22T</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KHRP26A33T</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KHRP26A72T</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KHRP26A73T</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>室內機分歧頭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BHFP22P100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BHFP22P151</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -12121,7 +12165,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F00506A-09F5-4009-80F2-281B4A4C3425}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:T20"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
@@ -12132,9 +12176,12 @@
     <col min="9" max="9" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.44140625" customWidth="1"/>
     <col min="12" max="12" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>569</v>
       </c>
@@ -12147,8 +12194,14 @@
       <c r="L1" t="s">
         <v>612</v>
       </c>
+      <c r="O1" t="s">
+        <v>557</v>
+      </c>
+      <c r="R1" t="s">
+        <v>626</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>605</v>
       </c>
@@ -12179,8 +12232,23 @@
       <c r="M2" t="s">
         <v>607</v>
       </c>
+      <c r="O2" t="s">
+        <v>605</v>
+      </c>
+      <c r="P2" t="s">
+        <v>607</v>
+      </c>
+      <c r="R2" t="s">
+        <v>605</v>
+      </c>
+      <c r="S2" t="s">
+        <v>607</v>
+      </c>
+      <c r="T2" t="s">
+        <v>610</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="61" t="s">
         <v>570</v>
       </c>
@@ -12211,8 +12279,23 @@
       <c r="M3">
         <v>4500</v>
       </c>
+      <c r="O3" t="s">
+        <v>561</v>
+      </c>
+      <c r="P3">
+        <v>4500</v>
+      </c>
+      <c r="R3" t="s">
+        <v>627</v>
+      </c>
+      <c r="S3">
+        <v>1700</v>
+      </c>
+      <c r="T3" t="s">
+        <v>631</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="61" t="s">
         <v>573</v>
       </c>
@@ -12237,8 +12320,17 @@
       <c r="J4">
         <v>1600</v>
       </c>
+      <c r="R4" t="s">
+        <v>628</v>
+      </c>
+      <c r="S4">
+        <v>2400</v>
+      </c>
+      <c r="T4" t="s">
+        <v>631</v>
+      </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>581</v>
       </c>
@@ -12254,8 +12346,17 @@
       <c r="J5">
         <v>1600</v>
       </c>
+      <c r="R5" t="s">
+        <v>629</v>
+      </c>
+      <c r="S5">
+        <v>3300</v>
+      </c>
+      <c r="T5" t="s">
+        <v>631</v>
+      </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="61" t="s">
         <v>574</v>
       </c>
@@ -12268,8 +12369,17 @@
       <c r="D6" t="s">
         <v>609</v>
       </c>
+      <c r="R6" t="s">
+        <v>630</v>
+      </c>
+      <c r="S6">
+        <v>4600</v>
+      </c>
+      <c r="T6" t="s">
+        <v>631</v>
+      </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>575</v>
       </c>
@@ -12279,8 +12389,17 @@
       <c r="C7">
         <v>7350</v>
       </c>
+      <c r="R7" t="s">
+        <v>632</v>
+      </c>
+      <c r="S7">
+        <v>3700</v>
+      </c>
+      <c r="T7" t="s">
+        <v>533</v>
+      </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="61" t="s">
         <v>578</v>
       </c>
@@ -12293,8 +12412,17 @@
       <c r="D8" t="s">
         <v>609</v>
       </c>
+      <c r="R8" t="s">
+        <v>633</v>
+      </c>
+      <c r="S8">
+        <v>7500</v>
+      </c>
+      <c r="T8" t="s">
+        <v>533</v>
+      </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>579</v>
       </c>
@@ -12305,7 +12433,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="61" t="s">
         <v>584</v>
       </c>
@@ -12320,7 +12448,7 @@
       </c>
       <c r="F10" s="62"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>586</v>
       </c>
@@ -12331,7 +12459,7 @@
         <v>28600</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>588</v>
       </c>
@@ -12342,7 +12470,7 @@
         <v>19400</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>591</v>
       </c>
@@ -12356,7 +12484,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>590</v>
       </c>
@@ -12367,7 +12495,7 @@
         <v>27500</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="61" t="s">
         <v>594</v>
       </c>
@@ -12381,7 +12509,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="61" t="s">
         <v>598</v>
       </c>
@@ -12429,6 +12557,21 @@
       </c>
       <c r="D19" t="s">
         <v>609</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="61" t="s">
+        <v>623</v>
+      </c>
+      <c r="B20" s="61" t="s">
+        <v>625</v>
+      </c>
+      <c r="C20">
+        <f>25350+2350</f>
+        <v>27700</v>
+      </c>
+      <c r="D20" t="s">
+        <v>624</v>
       </c>
     </row>
   </sheetData>

</xml_diff>